<commit_message>
fixed the alignment and template size
</commit_message>
<xml_diff>
--- a/email_log.xlsx
+++ b/email_log.xlsx
@@ -458,12 +458,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2025-03-27 21:33:51</t>
+          <t>2025-03-28 15:40:32</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>coder_akram.khan</t>
+          <t>WorkerSSal</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">

</xml_diff>